<commit_message>
added pricings to menu
</commit_message>
<xml_diff>
--- a/restaurant_menus.xlsx
+++ b/restaurant_menus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ooredoomle-my.sharepoint.com/personal/ahmed_maail_ooredoo_mv/Documents/vishaal idea/ramadan menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_F25DC773A252ABDACC1048D4395F6C085BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C62890B3-D242-4785-A771-2AF05D30AE9A}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="11_F25DC773A252ABDACC1048D4395F6C085BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{341788CB-D0EE-4A04-A7CE-14BE25915338}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="28">
   <si>
     <t>Day</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>monday</t>
+  </si>
+  <si>
+    <t>Price per Pax</t>
   </si>
 </sst>
 </file>
@@ -429,14 +432,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.42578125" customWidth="1"/>
     <col min="3" max="3" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,8 +449,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -457,8 +463,11 @@
       <c r="C2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -468,8 +477,11 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -479,8 +491,11 @@
       <c r="C4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -490,8 +505,11 @@
       <c r="C5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -501,8 +519,11 @@
       <c r="C6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -512,8 +533,11 @@
       <c r="C7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -523,8 +547,11 @@
       <c r="C8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -534,8 +561,11 @@
       <c r="C9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -545,8 +575,11 @@
       <c r="C10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -556,8 +589,11 @@
       <c r="C11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -567,8 +603,11 @@
       <c r="C12" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -578,8 +617,11 @@
       <c r="C13" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -589,8 +631,11 @@
       <c r="C14" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -600,8 +645,11 @@
       <c r="C15" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -611,8 +659,11 @@
       <c r="C16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -622,8 +673,11 @@
       <c r="C17" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -633,8 +687,11 @@
       <c r="C18" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -644,8 +701,11 @@
       <c r="C21" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -655,8 +715,11 @@
       <c r="C22" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -666,8 +729,11 @@
       <c r="C23" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -677,8 +743,11 @@
       <c r="C24" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -688,8 +757,11 @@
       <c r="C25" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -699,8 +771,11 @@
       <c r="C26" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -710,8 +785,11 @@
       <c r="C27" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -721,8 +799,11 @@
       <c r="C28" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -732,8 +813,11 @@
       <c r="C29" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -743,8 +827,11 @@
       <c r="C30" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
@@ -754,8 +841,11 @@
       <c r="C31" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -765,8 +855,11 @@
       <c r="C32" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D32">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>25</v>
       </c>
@@ -776,8 +869,11 @@
       <c r="C33" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D33">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>25</v>
       </c>
@@ -787,8 +883,11 @@
       <c r="C34" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -798,8 +897,11 @@
       <c r="C35" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -809,8 +911,11 @@
       <c r="C36" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D36">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -819,6 +924,9 @@
       </c>
       <c r="C37" t="s">
         <v>19</v>
+      </c>
+      <c r="D37">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added Acha's Poppadums menu
</commit_message>
<xml_diff>
--- a/restaurant_menus.xlsx
+++ b/restaurant_menus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ooredoomle-my.sharepoint.com/personal/ahmed_maail_ooredoo_mv/Documents/vishaal idea/ramadan menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="466" documentId="11_F25DC773A252ABDACC1048D4395F6C085BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AC237CA-34C0-41AA-91C3-DF74B507E2A3}"/>
+  <xr:revisionPtr revIDLastSave="656" documentId="11_F25DC773A252ABDACC1048D4395F6C085BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D2E78DA-3F94-4CF1-B02E-40F0315D2A15}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mamak" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="pomelo" sheetId="3" r:id="rId3"/>
     <sheet name="buruzu" sheetId="4" r:id="rId4"/>
     <sheet name="house of flavors" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
+    <sheet name="Acha's Poppadums" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2300" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2514" uniqueCount="271">
   <si>
     <t>Day</t>
   </si>
@@ -673,284 +674,194 @@
     <t>Aloo Gobi</t>
   </si>
   <si>
-    <t>Karaafani</t>
-  </si>
-  <si>
-    <t>Caesar Salad</t>
-  </si>
-  <si>
-    <t>Greek Salad</t>
-  </si>
-  <si>
-    <t>Roshi &amp; Battura</t>
-  </si>
-  <si>
-    <t>Mongolian Fried Rice</t>
-  </si>
-  <si>
-    <t>Penne Alfredo</t>
-  </si>
-  <si>
-    <t>Mustard Honey Chicken</t>
-  </si>
-  <si>
-    <t>Kan Kun Beef</t>
-  </si>
-  <si>
-    <t>Kulhi Mas</t>
-  </si>
-  <si>
-    <t>Aalu Gobi</t>
-  </si>
-  <si>
-    <t>Vegetable Chopsuey</t>
-  </si>
-  <si>
-    <t>Omaali</t>
-  </si>
-  <si>
-    <t>Blueberry Cheesecake</t>
-  </si>
-  <si>
-    <t>Assorted Fresh Fruits</t>
-  </si>
-  <si>
-    <t>Tea or Coffee</t>
-  </si>
-  <si>
-    <t>Water &amp; Nuts</t>
-  </si>
-  <si>
-    <t>Passionfruit Juice</t>
+    <t>FRIDAY</t>
+  </si>
+  <si>
+    <t>Drinks</t>
+  </si>
+  <si>
+    <t>Water melon</t>
+  </si>
+  <si>
+    <t>MVR 175+ GST</t>
+  </si>
+  <si>
+    <t>Mixed Fruit</t>
+  </si>
+  <si>
+    <t>Main Course</t>
+  </si>
+  <si>
+    <t>Schezwan Chicken</t>
+  </si>
+  <si>
+    <t>Beef Masala</t>
+  </si>
+  <si>
+    <t>Aalo Mutter</t>
+  </si>
+  <si>
+    <t>Tuna Noodles</t>
+  </si>
+  <si>
+    <t>Breads</t>
+  </si>
+  <si>
+    <t>Butter Naan</t>
+  </si>
+  <si>
+    <t>Paratta</t>
+  </si>
+  <si>
+    <t>Salad</t>
+  </si>
+  <si>
+    <t>Mixed Salad</t>
+  </si>
+  <si>
+    <t>Cut Fruits</t>
+  </si>
+  <si>
+    <t>Betel nuts</t>
+  </si>
+  <si>
+    <t>Tea/Coffee</t>
+  </si>
+  <si>
+    <t>Dessert</t>
+  </si>
+  <si>
+    <t>Rice Kheer</t>
+  </si>
+  <si>
+    <t>Gulab jamun</t>
+  </si>
+  <si>
+    <t>MONDAY</t>
+  </si>
+  <si>
+    <t>Pineapple</t>
+  </si>
+  <si>
+    <t>Chicken Fried Rice</t>
+  </si>
+  <si>
+    <t>Chicken Tikka Masala</t>
+  </si>
+  <si>
+    <t>Fish Manchurian</t>
+  </si>
+  <si>
+    <t>Mushroom &amp; Green peas</t>
+  </si>
+  <si>
+    <t>Masala</t>
+  </si>
+  <si>
+    <t>Beef Noodles</t>
+  </si>
+  <si>
+    <t>Roshi, Chapathi</t>
+  </si>
+  <si>
+    <t>Indian Garden Salad</t>
+  </si>
+  <si>
+    <t>Beetle nuts</t>
+  </si>
+  <si>
+    <t>Carrot Halwa</t>
+  </si>
+  <si>
+    <t>SATURDAY</t>
+  </si>
+  <si>
+    <t>Egg Noodles</t>
+  </si>
+  <si>
+    <t>Butter Chicken</t>
+  </si>
+  <si>
+    <t>Devilled Fish</t>
+  </si>
+  <si>
+    <t>Schezwan Chicken Rice</t>
+  </si>
+  <si>
+    <t>SUNDAY</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Beef Rogan josh</t>
+  </si>
+  <si>
+    <t>Aaloo Gobi Masala</t>
   </si>
   <si>
     <t>Green Salad</t>
   </si>
   <si>
-    <t>Roshi &amp; Fen Folhi</t>
-  </si>
-  <si>
-    <t>Macaroni Carbonara</t>
-  </si>
-  <si>
-    <t>Tandoori Chicken</t>
-  </si>
-  <si>
-    <t>Beef Bulgogi</t>
-  </si>
-  <si>
-    <t>Kandu Kukulhu</t>
-  </si>
-  <si>
-    <t>Sri Lankan Devilled Potato</t>
-  </si>
-  <si>
-    <t>Vegetable Manchurian</t>
-  </si>
-  <si>
-    <t>***************</t>
-  </si>
-  <si>
-    <t>Passion Fruit Mousse</t>
-  </si>
-  <si>
-    <t>Tiramisu Cake</t>
-  </si>
-  <si>
-    <t>Sweet Filling</t>
-  </si>
-  <si>
-    <t>Refreshments</t>
-  </si>
-  <si>
-    <t>大大火大大大大大大文大大大大大</t>
-  </si>
-  <si>
-    <t>Salads</t>
-  </si>
-  <si>
-    <t>Bashi Mas Huni</t>
-  </si>
-  <si>
-    <t>Chinese Fried Rice</t>
-  </si>
-  <si>
-    <t>Spaghetti Melanzane</t>
-  </si>
-  <si>
-    <t>Boot Stoganirt</t>
-  </si>
-  <si>
-    <t>Lebanese Grilled Chicken</t>
-  </si>
-  <si>
-    <t>HanaaKuri Mas</t>
-  </si>
-  <si>
-    <t>Tempered Potato</t>
-  </si>
-  <si>
-    <t>Cinnamon Cake with Ganache</t>
-  </si>
-  <si>
-    <t>Fruit Gateaux</t>
-  </si>
-  <si>
-    <t>Cheese Cake</t>
-  </si>
-  <si>
-    <t>*火大大大火大大大火大火大大大</t>
-  </si>
-  <si>
-    <t>Mango Juice</t>
-  </si>
-  <si>
-    <t>Thai Beef Salad</t>
-  </si>
-  <si>
-    <t>Roshi &amp; Fenfolhi</t>
-  </si>
-  <si>
-    <t>Spinach Fried Rice</t>
-  </si>
-  <si>
-    <t>Penne Alla Rustica</t>
-  </si>
-  <si>
-    <t>Chicken Tikka Masala</t>
-  </si>
-  <si>
-    <t>Lebanese Beef Kebab</t>
-  </si>
-  <si>
-    <t>Hanaakuri Mas</t>
-  </si>
-  <si>
-    <t>Hungarian Potato</t>
-  </si>
-  <si>
-    <t>Sauteed Vegetables</t>
-  </si>
-  <si>
-    <t>"******t"**</t>
-  </si>
-  <si>
-    <t>Le Lait Gateau</t>
-  </si>
-  <si>
-    <t>Cheese Cakae</t>
-  </si>
-  <si>
-    <t>Guava Juice</t>
-  </si>
-  <si>
-    <t>*************★*</t>
-  </si>
-  <si>
-    <t>American Salad</t>
-  </si>
-  <si>
-    <t>Maldivian Tuna Salad</t>
-  </si>
-  <si>
-    <t>Roshi &amp; Paratta</t>
-  </si>
-  <si>
-    <t>Manchurian Fried Rice</t>
-  </si>
-  <si>
-    <t>Spaghetti Bolognese</t>
-  </si>
-  <si>
-    <t>Alfaham Chicken</t>
-  </si>
-  <si>
-    <t>Srilankan Beef Curry</t>
-  </si>
-  <si>
-    <t>Grilled Fish Lemon Butter</t>
-  </si>
-  <si>
-    <t>Vegetable Au Gratin</t>
-  </si>
-  <si>
-    <t>**************</t>
-  </si>
-  <si>
-    <t>Kiwi Gateaux</t>
-  </si>
-  <si>
-    <t>Sweet Fling</t>
-  </si>
-  <si>
-    <t>Karaafani®</t>
-  </si>
-  <si>
-    <t>Thai Chicken Salad</t>
-  </si>
-  <si>
-    <t>Roshi &amp; Yeast Roshi</t>
-  </si>
-  <si>
-    <t>Sweet Corn &amp; Sultan Rice</t>
-  </si>
-  <si>
-    <t>Penne Alla Salsa Rosa</t>
-  </si>
-  <si>
-    <t>Tandoori Shish Kebab</t>
-  </si>
-  <si>
-    <t>Mongolian Beef</t>
-  </si>
-  <si>
-    <t>Musamma Curry</t>
-  </si>
-  <si>
-    <t>Aubergine Provencal</t>
-  </si>
-  <si>
-    <t>***%**********</t>
-  </si>
-  <si>
-    <t>Chocolate Mousse</t>
-  </si>
-  <si>
-    <t>Kesari</t>
-  </si>
-  <si>
-    <t>New York Cheesecake</t>
-  </si>
-  <si>
-    <t>****★**********</t>
-  </si>
-  <si>
-    <t>Florist Green Salad</t>
-  </si>
-  <si>
-    <t>Mixed Vegetable Pulao</t>
-  </si>
-  <si>
-    <t>Spaghetti Aglio Olio</t>
-  </si>
-  <si>
-    <t>Lebanese Chicken</t>
-  </si>
-  <si>
-    <t>Deviled Fish</t>
-  </si>
-  <si>
-    <t>**********w</t>
-  </si>
-  <si>
-    <t>Cinnamon Chocolate</t>
+    <t>Shahi Tukda</t>
+  </si>
+  <si>
+    <t>TUESDAY</t>
+  </si>
+  <si>
+    <t>Pappaya</t>
+  </si>
+  <si>
+    <t>Chicken Dopiyaza</t>
+  </si>
+  <si>
+    <t>Devilled Beef</t>
+  </si>
+  <si>
+    <t>Sweet n Sour Fish</t>
+  </si>
+  <si>
+    <t>Gobi Manchurian</t>
+  </si>
+  <si>
+    <t>Garlic Naan</t>
+  </si>
+  <si>
+    <t>Mixed Veg Salad</t>
+  </si>
+  <si>
+    <t>Semiya Kheer</t>
+  </si>
+  <si>
+    <t>WEDNESDAY</t>
+  </si>
+  <si>
+    <t>Beef Vindaloo</t>
+  </si>
+  <si>
+    <t>Garlic Fish</t>
+  </si>
+  <si>
+    <t>Paneer Butter Masala</t>
+  </si>
+  <si>
+    <t>THURSDAY</t>
+  </si>
+  <si>
+    <t>Veg Pulao</t>
+  </si>
+  <si>
+    <t>Chicken Kolhapuri</t>
+  </si>
+  <si>
+    <t>Aalo Gobi Capsicum</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -969,13 +880,6 @@
       <color theme="1"/>
       <name val="Helvetica"/>
       <family val="18"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -998,15 +902,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9076,992 +8977,1528 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C92B042-D4FF-2640-8B1F-B7EB4E9D16D9}">
-  <dimension ref="A1:D189"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60493718-0AF5-4082-ABAF-9F31032F6672}">
+  <dimension ref="A1:D134"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="A2" t="s">
         <v>210</v>
       </c>
-      <c r="D2">
-        <v>2</v>
+      <c r="B2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C3" s="2" t="s">
-        <v>7</v>
+      <c r="A3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2" t="s">
+      <c r="A4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B5" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>210</v>
+      </c>
+      <c r="B8" t="s">
+        <v>215</v>
+      </c>
+      <c r="C8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B9" t="s">
+        <v>215</v>
+      </c>
+      <c r="C9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" t="s">
+        <v>215</v>
+      </c>
+      <c r="C10" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>210</v>
+      </c>
+      <c r="B11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>210</v>
+      </c>
+      <c r="B12" t="s">
+        <v>220</v>
+      </c>
+      <c r="C12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" t="s">
+        <v>223</v>
+      </c>
+      <c r="C13" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>210</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B16" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
+      <c r="C16" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>210</v>
+      </c>
+      <c r="B18" t="s">
+        <v>211</v>
+      </c>
+      <c r="C18" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B19" t="s">
+        <v>228</v>
+      </c>
+      <c r="C19" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" t="s">
+        <v>228</v>
+      </c>
+      <c r="C20" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>231</v>
+      </c>
+      <c r="B21" t="s">
+        <v>211</v>
+      </c>
+      <c r="C21" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C7" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C8" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C9" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C10" s="2" t="s">
+      <c r="D21" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C11" s="2" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>231</v>
+      </c>
+      <c r="B22" t="s">
+        <v>211</v>
+      </c>
+      <c r="C22" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>231</v>
+      </c>
+      <c r="B23" t="s">
+        <v>215</v>
+      </c>
+      <c r="C23" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>231</v>
+      </c>
+      <c r="B24" t="s">
+        <v>215</v>
+      </c>
+      <c r="C24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>231</v>
+      </c>
+      <c r="B25" t="s">
+        <v>215</v>
+      </c>
+      <c r="C25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>231</v>
+      </c>
+      <c r="B26" t="s">
+        <v>215</v>
+      </c>
+      <c r="C26" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>231</v>
+      </c>
+      <c r="B27" t="s">
+        <v>215</v>
+      </c>
+      <c r="C27" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>231</v>
+      </c>
+      <c r="B28" t="s">
+        <v>215</v>
+      </c>
+      <c r="C28" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>231</v>
+      </c>
+      <c r="B29" t="s">
+        <v>215</v>
+      </c>
+      <c r="C29" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>231</v>
+      </c>
+      <c r="B30" t="s">
+        <v>220</v>
+      </c>
+      <c r="C30" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>231</v>
+      </c>
+      <c r="B31" t="s">
+        <v>220</v>
+      </c>
+      <c r="C31" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" t="s">
+        <v>223</v>
+      </c>
+      <c r="C32" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>231</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>231</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>231</v>
+      </c>
+      <c r="B35" t="s">
+        <v>211</v>
+      </c>
+      <c r="C35" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>231</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>231</v>
+      </c>
+      <c r="B37" t="s">
+        <v>211</v>
+      </c>
+      <c r="C37" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>231</v>
+      </c>
+      <c r="B38" t="s">
+        <v>228</v>
+      </c>
+      <c r="C38" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>231</v>
+      </c>
+      <c r="B39" t="s">
+        <v>228</v>
+      </c>
+      <c r="C39" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>243</v>
+      </c>
+      <c r="B40" t="s">
+        <v>211</v>
+      </c>
+      <c r="C40" t="s">
+        <v>212</v>
+      </c>
+      <c r="D40" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>243</v>
+      </c>
+      <c r="B41" t="s">
+        <v>211</v>
+      </c>
+      <c r="C41" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>243</v>
+      </c>
+      <c r="B42" t="s">
+        <v>215</v>
+      </c>
+      <c r="C42" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>243</v>
+      </c>
+      <c r="B43" t="s">
+        <v>215</v>
+      </c>
+      <c r="C43" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>243</v>
+      </c>
+      <c r="B44" t="s">
+        <v>215</v>
+      </c>
+      <c r="C44" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>243</v>
+      </c>
+      <c r="B45" t="s">
+        <v>215</v>
+      </c>
+      <c r="C45" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>243</v>
+      </c>
+      <c r="B46" t="s">
+        <v>215</v>
+      </c>
+      <c r="C46" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>243</v>
+      </c>
+      <c r="B47" t="s">
+        <v>215</v>
+      </c>
+      <c r="C47" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>243</v>
+      </c>
+      <c r="B48" t="s">
+        <v>220</v>
+      </c>
+      <c r="C48" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>243</v>
+      </c>
+      <c r="B49" t="s">
+        <v>220</v>
+      </c>
+      <c r="C49" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>243</v>
+      </c>
+      <c r="B50" t="s">
+        <v>220</v>
+      </c>
+      <c r="C50" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>243</v>
+      </c>
+      <c r="B51" t="s">
+        <v>223</v>
+      </c>
+      <c r="C51" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>243</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>243</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>243</v>
+      </c>
+      <c r="B54" t="s">
+        <v>211</v>
+      </c>
+      <c r="C54" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>243</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>243</v>
+      </c>
+      <c r="B56" t="s">
+        <v>211</v>
+      </c>
+      <c r="C56" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>243</v>
+      </c>
+      <c r="B57" t="s">
+        <v>228</v>
+      </c>
+      <c r="C57" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>243</v>
+      </c>
+      <c r="B58" t="s">
+        <v>228</v>
+      </c>
+      <c r="C58" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>248</v>
+      </c>
+      <c r="B59" t="s">
+        <v>211</v>
+      </c>
+      <c r="C59" t="s">
+        <v>212</v>
+      </c>
+      <c r="D59" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>248</v>
+      </c>
+      <c r="B60" t="s">
+        <v>211</v>
+      </c>
+      <c r="C60" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>248</v>
+      </c>
+      <c r="B61" t="s">
+        <v>215</v>
+      </c>
+      <c r="C61" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>248</v>
+      </c>
+      <c r="B62" t="s">
+        <v>215</v>
+      </c>
+      <c r="C62" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>248</v>
+      </c>
+      <c r="B63" t="s">
+        <v>215</v>
+      </c>
+      <c r="C63" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>248</v>
+      </c>
+      <c r="B64" t="s">
+        <v>215</v>
+      </c>
+      <c r="C64" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>248</v>
+      </c>
+      <c r="B65" t="s">
+        <v>215</v>
+      </c>
+      <c r="C65" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>248</v>
+      </c>
+      <c r="B66" t="s">
+        <v>215</v>
+      </c>
+      <c r="C66" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>248</v>
+      </c>
+      <c r="B67" t="s">
+        <v>220</v>
+      </c>
+      <c r="C67" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>248</v>
+      </c>
+      <c r="B68" t="s">
+        <v>220</v>
+      </c>
+      <c r="C68" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>248</v>
+      </c>
+      <c r="B69" t="s">
+        <v>223</v>
+      </c>
+      <c r="C69" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>248</v>
+      </c>
+      <c r="B70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>248</v>
+      </c>
+      <c r="B71" t="s">
+        <v>8</v>
+      </c>
+      <c r="C71" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>248</v>
+      </c>
+      <c r="B72" t="s">
+        <v>211</v>
+      </c>
+      <c r="C72" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>248</v>
+      </c>
+      <c r="B73" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>248</v>
+      </c>
+      <c r="B74" t="s">
+        <v>211</v>
+      </c>
+      <c r="C74" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>248</v>
+      </c>
+      <c r="B75" t="s">
+        <v>228</v>
+      </c>
+      <c r="C75" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>248</v>
+      </c>
+      <c r="B76" t="s">
+        <v>228</v>
+      </c>
+      <c r="C76" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>254</v>
+      </c>
+      <c r="B77" t="s">
+        <v>211</v>
+      </c>
+      <c r="C77" t="s">
+        <v>212</v>
+      </c>
+      <c r="D77" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>254</v>
+      </c>
+      <c r="B78" t="s">
+        <v>211</v>
+      </c>
+      <c r="C78" t="s">
+        <v>255</v>
+      </c>
+      <c r="D78" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>254</v>
+      </c>
+      <c r="B79" t="s">
+        <v>215</v>
+      </c>
+      <c r="C79" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>254</v>
+      </c>
+      <c r="B80" t="s">
+        <v>215</v>
+      </c>
+      <c r="C80" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>254</v>
+      </c>
+      <c r="B81" t="s">
+        <v>215</v>
+      </c>
+      <c r="C81" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>254</v>
+      </c>
+      <c r="B82" t="s">
+        <v>215</v>
+      </c>
+      <c r="C82" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>254</v>
+      </c>
+      <c r="B83" t="s">
+        <v>215</v>
+      </c>
+      <c r="C83" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>254</v>
+      </c>
+      <c r="B84" t="s">
+        <v>215</v>
+      </c>
+      <c r="C84" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>254</v>
+      </c>
+      <c r="B85" t="s">
+        <v>215</v>
+      </c>
+      <c r="C85" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>254</v>
+      </c>
+      <c r="B86" t="s">
+        <v>220</v>
+      </c>
+      <c r="C86" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>254</v>
+      </c>
+      <c r="B87" t="s">
+        <v>220</v>
+      </c>
+      <c r="C87" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>254</v>
+      </c>
+      <c r="B88" t="s">
+        <v>223</v>
+      </c>
+      <c r="C88" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>254</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>254</v>
+      </c>
+      <c r="B90" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>254</v>
+      </c>
+      <c r="B91" t="s">
+        <v>211</v>
+      </c>
+      <c r="C91" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>254</v>
+      </c>
+      <c r="B92" t="s">
+        <v>8</v>
+      </c>
+      <c r="C92" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>254</v>
+      </c>
+      <c r="B93" t="s">
+        <v>211</v>
+      </c>
+      <c r="C93" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>254</v>
+      </c>
+      <c r="B94" t="s">
+        <v>228</v>
+      </c>
+      <c r="C94" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>254</v>
+      </c>
+      <c r="B95" t="s">
+        <v>228</v>
+      </c>
+      <c r="C95" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>263</v>
+      </c>
+      <c r="B96" t="s">
+        <v>211</v>
+      </c>
+      <c r="C96" t="s">
+        <v>212</v>
+      </c>
+      <c r="D96" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>263</v>
+      </c>
+      <c r="B97" t="s">
+        <v>211</v>
+      </c>
+      <c r="C97" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C12" s="2" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>263</v>
+      </c>
+      <c r="B98" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C13" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C14" s="2" t="s">
+      <c r="C98" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>263</v>
+      </c>
+      <c r="B99" t="s">
+        <v>215</v>
+      </c>
+      <c r="C99" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>263</v>
+      </c>
+      <c r="B100" t="s">
+        <v>215</v>
+      </c>
+      <c r="C100" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>263</v>
+      </c>
+      <c r="B101" t="s">
+        <v>215</v>
+      </c>
+      <c r="C101" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>263</v>
+      </c>
+      <c r="B102" t="s">
+        <v>215</v>
+      </c>
+      <c r="C102" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>263</v>
+      </c>
+      <c r="B103" t="s">
+        <v>215</v>
+      </c>
+      <c r="C103" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>263</v>
+      </c>
+      <c r="B104" t="s">
+        <v>215</v>
+      </c>
+      <c r="C104" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>263</v>
+      </c>
+      <c r="B105" t="s">
+        <v>220</v>
+      </c>
+      <c r="C105" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>263</v>
+      </c>
+      <c r="B106" t="s">
+        <v>220</v>
+      </c>
+      <c r="C106" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>263</v>
+      </c>
+      <c r="B107" t="s">
+        <v>223</v>
+      </c>
+      <c r="C107" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>263</v>
+      </c>
+      <c r="B108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C108" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>263</v>
+      </c>
+      <c r="B109" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>263</v>
+      </c>
+      <c r="B110" t="s">
+        <v>211</v>
+      </c>
+      <c r="C110" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>263</v>
+      </c>
+      <c r="B111" t="s">
+        <v>8</v>
+      </c>
+      <c r="C111" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>263</v>
+      </c>
+      <c r="B112" t="s">
+        <v>211</v>
+      </c>
+      <c r="C112" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>263</v>
+      </c>
+      <c r="B113" t="s">
+        <v>228</v>
+      </c>
+      <c r="C113" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>263</v>
+      </c>
+      <c r="B114" t="s">
+        <v>228</v>
+      </c>
+      <c r="C114" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>267</v>
+      </c>
+      <c r="B115" t="s">
+        <v>211</v>
+      </c>
+      <c r="C115" t="s">
+        <v>212</v>
+      </c>
+      <c r="D115" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>267</v>
+      </c>
+      <c r="B116" t="s">
+        <v>211</v>
+      </c>
+      <c r="C116" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>267</v>
+      </c>
+      <c r="B117" t="s">
+        <v>215</v>
+      </c>
+      <c r="C117" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>267</v>
+      </c>
+      <c r="B118" t="s">
+        <v>215</v>
+      </c>
+      <c r="C118" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>267</v>
+      </c>
+      <c r="B119" t="s">
+        <v>215</v>
+      </c>
+      <c r="C119" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C15" s="2" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C16" s="2" t="s">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>267</v>
+      </c>
+      <c r="B120" t="s">
+        <v>215</v>
+      </c>
+      <c r="C120" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>267</v>
+      </c>
+      <c r="B121" t="s">
+        <v>215</v>
+      </c>
+      <c r="C121" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>267</v>
+      </c>
+      <c r="B122" t="s">
+        <v>215</v>
+      </c>
+      <c r="C122" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>267</v>
+      </c>
+      <c r="B123" t="s">
+        <v>215</v>
+      </c>
+      <c r="C123" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>267</v>
+      </c>
+      <c r="B124" t="s">
+        <v>215</v>
+      </c>
+      <c r="C124" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="2" t="s">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>267</v>
+      </c>
+      <c r="B125" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C18" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C19" s="2" t="s">
+      <c r="C125" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C20" s="2" t="s">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>267</v>
+      </c>
+      <c r="B126" t="s">
+        <v>220</v>
+      </c>
+      <c r="C126" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C21" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C22" s="2" t="s">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>267</v>
+      </c>
+      <c r="B127" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C24" s="2" t="s">
+      <c r="C127" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>267</v>
+      </c>
+      <c r="B128" t="s">
+        <v>8</v>
+      </c>
+      <c r="C128" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="2" t="s">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>267</v>
+      </c>
+      <c r="B129" t="s">
+        <v>8</v>
+      </c>
+      <c r="C129" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>267</v>
+      </c>
+      <c r="B130" t="s">
+        <v>211</v>
+      </c>
+      <c r="C130" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>267</v>
+      </c>
+      <c r="B131" t="s">
+        <v>8</v>
+      </c>
+      <c r="C131" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="2" t="s">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>267</v>
+      </c>
+      <c r="B132" t="s">
+        <v>211</v>
+      </c>
+      <c r="C132" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C30" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C31" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C32" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C34" s="2" t="s">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>267</v>
+      </c>
+      <c r="B133" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C37" s="2" t="s">
+      <c r="C133" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>267</v>
+      </c>
+      <c r="B134" t="s">
+        <v>228</v>
+      </c>
+      <c r="C134" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C38" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C39" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C40" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C41" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C42" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C45" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C48" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C50" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C52" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="24.75" x14ac:dyDescent="0.25">
-      <c r="C54" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C56" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C58" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C59" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C60" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C61" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C62" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C63" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C64" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C73" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C74" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C75" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C76" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C77" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C78" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="24.75" x14ac:dyDescent="0.25">
-      <c r="A79" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C80" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C81" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C82" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C83" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C84" s="2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="85" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C85" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="86" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C86" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="87" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C87" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="88" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C88" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="89" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C89" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="90" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C90" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="91" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C91" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="92" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C92" s="2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="93" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C93" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="94" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C94" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="95" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C95" s="2" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="96" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C96" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C97" s="2" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C98" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C99" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C100" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C101" s="2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C102" s="2" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C103" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C104" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C105" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C106" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C108" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C109" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C110" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C111" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C112" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="113" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C113" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="114" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C114" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="115" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C115" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="116" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C116" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="117" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C117" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="118" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C118" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="119" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C119" s="2" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="120" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C120" s="2" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="121" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C121" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="122" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C122" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="123" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C123" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="124" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C124" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="125" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C125" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="126" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C126" s="2" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="127" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C127" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="128" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C128" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C129" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C130" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C131" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C132" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C133" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C134" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A135" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C136" s="2" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C137" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C138" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C139" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C140" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C141" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C142" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C143" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C144" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="145" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C145" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="146" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C146" s="2" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="147" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C147" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="148" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C148" s="2" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="149" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C149" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="150" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C150" s="2" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="151" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C151" s="2" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="152" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C152" s="2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="153" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C153" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="154" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C154" s="2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="155" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C155" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="156" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C156" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="157" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C157" s="2" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="158" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C158" s="2" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="159" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C159" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="160" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C160" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C161" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C162" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C163" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C164" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C165" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C166" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C167" s="2" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C168" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C169" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C170" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C171" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C172" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C173" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C174" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C175" s="2" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C176" s="2" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="177" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C177" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="178" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C178" s="2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="179" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C179" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="180" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C180" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="181" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C181" s="2" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="182" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C182" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="183" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C183" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="184" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C184" s="2" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="185" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C185" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="186" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C186" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="187" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C187" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="188" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C188" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="189" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C189" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91C3AD69-3D4C-4C60-8E1B-122A3BE35217}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>